<commit_message>
Added default options for direct trajectory conversion
</commit_message>
<xml_diff>
--- a/data/empty_dataset.xlsx
+++ b/data/empty_dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UserData\TERCOM\TERCOM_py\SPS-main\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Standardnutzer\source\repos\SPS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9C07291-5BCE-45E4-956F-E8DBD4482354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E968007F-44EE-4EF7-BC82-669153204B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{E459F509-91DB-4780-AC17-CE2B8D072DEC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Name</t>
   </si>
@@ -60,27 +60,6 @@
   </si>
   <si>
     <t>TAEPO</t>
-  </si>
-  <si>
-    <t>body_1</t>
-  </si>
-  <si>
-    <t>1e28</t>
-  </si>
-  <si>
-    <t>1.5e11</t>
-  </si>
-  <si>
-    <t>0.0</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>0.8</t>
   </si>
 </sst>
 </file>
@@ -453,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A541A9-2EF5-4677-A83F-A2E52C7F45D8}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="16384" width="11.453125" style="1"/>
@@ -485,32 +464,6 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
MY WAS CHANGED BEWARE
</commit_message>
<xml_diff>
--- a/data/empty_dataset.xlsx
+++ b/data/empty_dataset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Standardnutzer\source\repos\SPS\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Non-Admin\source\repos\Orbital Mechanics\SPS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E968007F-44EE-4EF7-BC82-669153204B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4BBEB67-71CE-4E11-8DCD-60BD8954C5CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{E459F509-91DB-4780-AC17-CE2B8D072DEC}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11385" xr2:uid="{E459F509-91DB-4780-AC17-CE2B8D072DEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -433,12 +433,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A541A9-2EF5-4677-A83F-A2E52C7F45D8}">
   <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.453125" style="1"/>
+    <col min="1" max="1" width="11.42578125" style="1"/>
+    <col min="2" max="2" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>